<commit_message>
chore: add brand assets, agent skills, scripts, audit docs & project files
- add generated brand/favicon/logo/qr assets and brand shared component
- add agent security-testing skills (.agents) and scripts (brand asset sync)
- add audit docs, referenceScripts, refresh-mcp-token utility
- add source (propaura.cdr) plus backup, propaura.md, skills-lock
- remove obsolete root svg assets; refresh Rent_Data_Template xlsx and routes
</commit_message>
<xml_diff>
--- a/Rent_Data_Template (14).xlsx
+++ b/Rent_Data_Template (14).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VEGA\RENT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A44DB45B-C816-4389-8F82-25701C2D966A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F0975E-DC5C-4E51-AA34-85913C91E9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tenant_Profile" sheetId="1" r:id="rId1"/>
@@ -29,15 +29,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
   <si>
     <t>Phone</t>
   </si>
@@ -148,13 +145,16 @@
   </si>
   <si>
     <t>tankWater</t>
+  </si>
+  <si>
+    <t>T1-002</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,6 +167,12 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -567,7 +573,7 @@
         <v>24</v>
       </c>
       <c r="C2">
-        <v>9599130381</v>
+        <v>8389095941</v>
       </c>
       <c r="G2" t="s">
         <v>25</v>
@@ -604,10 +610,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -732,7 +738,67 @@
         <v>23</v>
       </c>
     </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46204</v>
+      </c>
+      <c r="D3" s="3">
+        <v>46235</v>
+      </c>
+      <c r="E3">
+        <v>600</v>
+      </c>
+      <c r="F3">
+        <v>720</v>
+      </c>
+      <c r="G3">
+        <f>F3-E3</f>
+        <v>120</v>
+      </c>
+      <c r="H3">
+        <v>8000</v>
+      </c>
+      <c r="I3">
+        <v>500</v>
+      </c>
+      <c r="J3">
+        <f>G3*Tenant_Profile!L3</f>
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>1250</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <f>SUM(H3:N3)</f>
+        <v>9750</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>26</v>
+      </c>
+      <c r="R3" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>